<commit_message>
24-8 vardiyasi 24.00 oncesi diger gune kaydedilmesi gerceklestirildi
</commit_message>
<xml_diff>
--- a/data/Fide_Konserve_Gunluk_Bolum_Calisan_Sayilari_Eylül_2026.xlsx
+++ b/data/Fide_Konserve_Gunluk_Bolum_Calisan_Sayilari_Eylül_2026.xlsx
@@ -918,7 +918,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>KALİTE</t>
+          <t>BAKIM</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -1067,20 +1067,20 @@
         </is>
       </c>
       <c r="AF5" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG5" s="11">
         <f>SUM(C5:AF5)</f>
         <v/>
       </c>
       <c r="AH5" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AI5" s="13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AJ5" s="14" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>BAKIM</t>
+          <t>KALİTE</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -1238,20 +1238,20 @@
         </is>
       </c>
       <c r="AF6" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG6" s="11">
         <f>SUM(C6:AF6)</f>
         <v/>
       </c>
       <c r="AH6" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI6" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AJ6" s="14" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>KAPI GÖREVLİSİ</t>
+          <t>AMBAR</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -1409,20 +1409,20 @@
         </is>
       </c>
       <c r="AF7" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG7" s="11">
         <f>SUM(C7:AF7)</f>
         <v/>
       </c>
       <c r="AH7" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI7" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ7" s="14" t="n">
-        <v>15</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="8">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>AMBAR</t>
+          <t>ELEKTRİK</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>ELEKTRİK</t>
+          <t>GENEL</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -1705,10 +1705,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W9" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="W9" s="15" t="n">
+        <v>1</v>
       </c>
       <c r="X9" s="8" t="inlineStr">
         <is>
@@ -1750,8 +1748,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AF9" s="15" t="n">
-        <v>1</v>
+      <c r="AF9" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AG9" s="11">
         <f>SUM(C9:AF9)</f>
@@ -1764,7 +1764,7 @@
         <v>1</v>
       </c>
       <c r="AJ9" s="14" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="10">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>GENEL</t>
+          <t>KAPI GÖREVLİSİ</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -1876,53 +1876,53 @@
           <t>-</t>
         </is>
       </c>
-      <c r="W10" s="15" t="n">
+      <c r="W10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC10" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF10" s="15" t="n">
         <v>1</v>
-      </c>
-      <c r="X10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AC10" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
       </c>
       <c r="AG10" s="11">
         <f>SUM(C10:AF10)</f>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>MEYDAN</t>
+          <t>OTOKLAV OPERATÖRÜ</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>OTOKLAV OPERATÖRÜ</t>
+          <t>YEMEKHANE</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -2448,7 +2448,7 @@
         <v>1</v>
       </c>
       <c r="AJ13" s="14" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="14">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>YEMEKHANE</t>
+          <t>İŞLETME</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -2619,7 +2619,7 @@
         <v>1</v>
       </c>
       <c r="AJ14" s="14" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="15">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>YENİ BALIK HATTI</t>
+          <t>BALIK</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -2776,21 +2776,23 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AF15" s="15" t="n">
-        <v>1</v>
+      <c r="AF15" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AG15" s="11">
         <f>SUM(C15:AF15)</f>
         <v/>
       </c>
       <c r="AH15" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI15" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ15" s="14" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -2799,7 +2801,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>İŞLETME</t>
+          <t>BALIK DOLUM</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -2947,21 +2949,23 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AF16" s="15" t="n">
-        <v>1</v>
+      <c r="AF16" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AG16" s="11">
         <f>SUM(C16:AF16)</f>
         <v/>
       </c>
       <c r="AH16" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI16" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ16" s="14" t="n">
-        <v>10.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -2970,7 +2974,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>ŞÖFÖR</t>
+          <t>BALIK KESİM</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -3118,21 +3122,23 @@
           <t>-</t>
         </is>
       </c>
-      <c r="AF17" s="15" t="n">
-        <v>1</v>
+      <c r="AF17" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AG17" s="11">
         <f>SUM(C17:AF17)</f>
         <v/>
       </c>
       <c r="AH17" s="12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI17" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ17" s="14" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3141,7 +3147,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>BALIK</t>
+          <t>BALIK TEMİZLEME</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -3314,7 +3320,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>BALIK DOLUM</t>
+          <t>BALIK TEMİZLİK</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -3487,7 +3493,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>BALIK KESİM</t>
+          <t>BİLGİSAYAR MÜHENDİSİ</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
@@ -3660,7 +3666,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>BALIK TEMİZLEME</t>
+          <t>DİĞER</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -3833,7 +3839,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>BALIK TEMİZLİK</t>
+          <t>FAB.MD</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -4006,7 +4012,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>BİLGİSAYAR MÜHENDİSİ</t>
+          <t>FORMEN</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -4179,7 +4185,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>DİĞER</t>
+          <t>KONSERVE ÜRETİM ELEMANI</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -4352,7 +4358,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>FAB.MD</t>
+          <t>MEYDAN</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -4525,7 +4531,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>FORMEN</t>
+          <t>MUHASEBE</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -4698,7 +4704,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>KONSERVE ÜRETİM ELEMANI</t>
+          <t>SATIN ALMA</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -4871,7 +4877,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>MUHASEBE</t>
+          <t>YENİ BALIK HATTI</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -5044,7 +5050,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>SATIN ALMA</t>
+          <t>ÇEVRE MÜHENDİSİ</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -5217,7 +5223,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>ÇEVRE MÜHENDİSİ</t>
+          <t>İNSAN KAYNAKLARI</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
@@ -5390,7 +5396,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>İNSAN KAYNAKLARI</t>
+          <t>ŞÖFÖR</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -5715,7 +5721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5862,7 +5868,7 @@
       </c>
       <c r="J3" s="22" t="inlineStr">
         <is>
-          <t>%40.0</t>
+          <t>%52.2</t>
         </is>
       </c>
     </row>
@@ -5887,24 +5893,24 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>KALİTE</t>
+          <t>BAKIM</t>
         </is>
       </c>
       <c r="F4" s="22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G4" s="22" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="H4" s="22" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="I4" s="22" t="n">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="J4" s="22" t="inlineStr">
         <is>
-          <t>%13.3</t>
+          <t>%8.7</t>
         </is>
       </c>
     </row>
@@ -5929,24 +5935,24 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>BAKIM</t>
+          <t>KALİTE</t>
         </is>
       </c>
       <c r="F5" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="H5" s="22" t="n">
-        <v>3.5</v>
+        <v>0.5</v>
       </c>
       <c r="I5" s="22" t="n">
-        <v>8.699999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="J5" s="22" t="inlineStr">
         <is>
-          <t>%10.0</t>
+          <t>%8.7</t>
         </is>
       </c>
     </row>
@@ -5971,24 +5977,24 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>KAPI GÖREVLİSİ</t>
+          <t>AMBAR</t>
         </is>
       </c>
       <c r="F6" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>15</v>
+        <v>10.5</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>7.5</v>
+        <v>10.5</v>
       </c>
       <c r="J6" s="22" t="inlineStr">
         <is>
-          <t>%6.7</t>
+          <t>%4.3</t>
         </is>
       </c>
     </row>
@@ -6013,7 +6019,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>AMBAR</t>
+          <t>ELEKTRİK</t>
         </is>
       </c>
       <c r="F7" s="22" t="n">
@@ -6030,7 +6036,7 @@
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>%3.3</t>
+          <t>%4.3</t>
         </is>
       </c>
     </row>
@@ -6055,24 +6061,24 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>ELEKTRİK</t>
+          <t>KAPI GÖREVLİSİ</t>
         </is>
       </c>
       <c r="F8" s="22" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
       <c r="J8" s="22" t="inlineStr">
         <is>
-          <t>%3.3</t>
+          <t>%4.3</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6120,7 @@
       </c>
       <c r="J9" s="22" t="inlineStr">
         <is>
-          <t>%3.3</t>
+          <t>%4.3</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6145,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>MEYDAN</t>
+          <t>OTOKLAV OPERATÖRÜ</t>
         </is>
       </c>
       <c r="F10" s="22" t="n">
@@ -6156,7 +6162,7 @@
       </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
-          <t>%3.3</t>
+          <t>%4.3</t>
         </is>
       </c>
     </row>
@@ -6181,24 +6187,24 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>OTOKLAV OPERATÖRÜ</t>
+          <t>YEMEKHANE</t>
         </is>
       </c>
       <c r="F11" s="22" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="22" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" s="22" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="J11" s="22" t="inlineStr">
         <is>
-          <t>%3.3</t>
+          <t>%4.3</t>
         </is>
       </c>
     </row>
@@ -6223,150 +6229,24 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>YEMEKHANE</t>
+          <t>İŞLETME</t>
         </is>
       </c>
       <c r="F12" s="22" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="22" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="J12" s="22" t="inlineStr">
         <is>
-          <t>%3.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>30.09.2026</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Çarşamba</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Hafta İçi</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>YENİ BALIK HATTI</t>
-        </is>
-      </c>
-      <c r="F13" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="22" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="H13" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="22" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="J13" s="22" t="inlineStr">
-        <is>
-          <t>%3.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>30.09.2026</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Çarşamba</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Hafta İçi</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>İŞLETME</t>
-        </is>
-      </c>
-      <c r="F14" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="22" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H14" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="I14" s="22" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="J14" s="22" t="inlineStr">
-        <is>
-          <t>%3.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>30.09.2026</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Çarşamba</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Hafta İçi</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>ŞÖFÖR</t>
-        </is>
-      </c>
-      <c r="F15" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="22" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="H15" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="22" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="J15" s="22" t="inlineStr">
-        <is>
-          <t>%3.3</t>
+          <t>%4.3</t>
         </is>
       </c>
     </row>

</xml_diff>